<commit_message>
Add 5 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 28
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-detail.report.xlsx
+++ b/tools/importer/reports/import-article-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="287">
   <si>
     <t>_reportFile</t>
   </si>
@@ -152,6 +152,252 @@
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumbs","carousel","tabs"]</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:13:49.974Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:13:55.313Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:13:59.987Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:04.575Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:08.288Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:14.305Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:19.715Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:25.358Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:29.824Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:36.070Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:42.054Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:46.494Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:51.889Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:14:57.107Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:15:02.508Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-18T17:15:07.400Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/yosemite-backpacking.html</t>
   </si>
   <si>
     <t>us/en/adventures/bali-surf-camp.html.report.json</t>
@@ -184,19 +430,10 @@
     <t>us/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
-    <t>["carousel","columns"]</t>
-  </si>
-  <si>
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>adventure-detail</t>
-  </si>
-  <si>
-    <t>2026-09-16T17:00:57.404Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
+    <t>2026-09-18T17:15:13.088Z</t>
   </si>
   <si>
     <t>us/en/adventures/beervana-portland.html.report.json</t>
@@ -217,10 +454,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:02.720Z</t>
-  </si>
-  <si>
-    <t>Beervana in Portland</t>
+    <t>2026-09-18T17:15:17.953Z</t>
   </si>
   <si>
     <t>us/en/adventures/climbing-new-zealand.html.report.json</t>
@@ -241,10 +475,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-16T17:00:52.532Z</t>
-  </si>
-  <si>
-    <t>Climbing New Zealand</t>
+    <t>2026-09-18T17:15:24.088Z</t>
   </si>
   <si>
     <t>us/en/adventures/colorado-rock-climbing.html.report.json</t>
@@ -265,10 +496,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:06.904Z</t>
-  </si>
-  <si>
-    <t>Colorado Rock Climbing</t>
+    <t>2026-09-18T17:15:29.088Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-southern-utah.html.report.json</t>
@@ -289,10 +517,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:11.049Z</t>
-  </si>
-  <si>
-    <t>Cycling Southern Utah</t>
+    <t>2026-09-18T17:15:33.231Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-tuscany.html.report.json</t>
@@ -313,10 +538,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:15.821Z</t>
-  </si>
-  <si>
-    <t>Cycling Tuscany</t>
+    <t>2026-09-18T17:15:39.061Z</t>
   </si>
   <si>
     <t>us/en/adventures/downhill-skiing-wyoming.html.report.json</t>
@@ -337,10 +559,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:20.932Z</t>
-  </si>
-  <si>
-    <t>Downhill Skiing Wyoming</t>
+    <t>2026-09-18T17:15:44.532Z</t>
   </si>
   <si>
     <t>us/en/adventures/gastronomic-marais-tour.html.report.json</t>
@@ -361,10 +580,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:25.413Z</t>
-  </si>
-  <si>
-    <t>Gastronomic Marais Tour</t>
+    <t>2026-09-18T17:15:48.415Z</t>
   </si>
   <si>
     <t>us/en/adventures/napa-wine-tasting.html.report.json</t>
@@ -385,10 +601,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:31.236Z</t>
-  </si>
-  <si>
-    <t>Napa Wine Tasting</t>
+    <t>2026-09-18T17:15:53.895Z</t>
   </si>
   <si>
     <t>us/en/adventures/riverside-camping-australia.html.report.json</t>
@@ -409,10 +622,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:35.317Z</t>
-  </si>
-  <si>
-    <t>Riverside Camping</t>
+    <t>2026-09-18T17:16:00.077Z</t>
   </si>
   <si>
     <t>us/en/adventures/ski-touring-mont-blanc.html.report.json</t>
@@ -433,10 +643,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:40.653Z</t>
-  </si>
-  <si>
-    <t>Ski Touring Mont Blanc</t>
+    <t>2026-09-18T17:16:04.133Z</t>
   </si>
   <si>
     <t>us/en/adventures/surf-camp-costa-rica.html.report.json</t>
@@ -457,10 +664,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:45.264Z</t>
-  </si>
-  <si>
-    <t>Surf Camp in Costa Rica</t>
+    <t>2026-09-18T17:16:07.950Z</t>
   </si>
   <si>
     <t>us/en/adventures/tahoe-skiing.html.report.json</t>
@@ -481,10 +685,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:50.791Z</t>
-  </si>
-  <si>
-    <t>Tahoe Skiing</t>
+    <t>2026-09-18T17:16:12.574Z</t>
   </si>
   <si>
     <t>us/en/adventures/west-coast-cycling.html.report.json</t>
@@ -505,10 +706,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-16T17:01:56.295Z</t>
-  </si>
-  <si>
-    <t>West Coast Cycling</t>
+    <t>2026-09-18T17:16:17.884Z</t>
   </si>
   <si>
     <t>us/en/adventures/whistler-mountain-biking.html.report.json</t>
@@ -529,10 +727,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:01.942Z</t>
-  </si>
-  <si>
-    <t>Whistler Mountain Biking</t>
+    <t>2026-09-18T17:16:22.722Z</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking.html.report.json</t>
@@ -553,10 +748,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:08.070Z</t>
-  </si>
-  <si>
-    <t>Yosemite Backpacking</t>
+    <t>2026-09-18T17:16:27.596Z</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing.html.report.json</t>
@@ -628,10 +820,13 @@
     <t>us/en/magazine/san-diego-surf.report.json</t>
   </si>
   <si>
+    <t>["hero-article","breadcrumbs","author-bio","author-bio","cards-related"]</t>
+  </si>
+  <si>
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:24.085Z</t>
+    <t>2026-09-18T17:55:40.644Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -1071,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1278,28 +1473,28 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
         <v>49</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
         <v>50</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>51</v>
       </c>
-      <c r="G7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>52</v>
-      </c>
-      <c r="I7" t="s">
-        <v>12</v>
       </c>
       <c r="J7" t="s">
         <v>53</v>
@@ -1310,60 +1505,60 @@
         <v>54</v>
       </c>
       <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
         <v>55</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
         <v>56</v>
       </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>57</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>58</v>
-      </c>
-      <c r="I8" t="s">
-        <v>59</v>
-      </c>
-      <c r="J8" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
         <v>61</v>
       </c>
-      <c r="F9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>62</v>
-      </c>
-      <c r="I9" t="s">
-        <v>12</v>
       </c>
       <c r="J9" t="s">
         <v>63</v>
@@ -1374,7 +1569,7 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1389,7 +1584,7 @@
         <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H10" t="s">
         <v>66</v>
@@ -1398,47 +1593,47 @@
         <v>67</v>
       </c>
       <c r="J10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I11" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1447,62 +1642,62 @@
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F13" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I13" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="J13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1511,62 +1706,62 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="J14" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H15" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="I15" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1575,62 +1770,62 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H16" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="J16" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I17" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="J17" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -1639,62 +1834,62 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="I18" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="J18" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="F19" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="I19" t="s">
-        <v>12</v>
+        <v>112</v>
       </c>
       <c r="J19" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1703,62 +1898,62 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I20" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="J20" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H21" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="I21" t="s">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="J21" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1767,62 +1962,62 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H22" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="I22" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="J22" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E23" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="F23" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G23" t="s">
         <v>12</v>
       </c>
       <c r="H23" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="I23" t="s">
         <v>12</v>
       </c>
       <c r="J23" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -1831,62 +2026,62 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H24" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="I24" t="s">
-        <v>123</v>
+        <v>52</v>
       </c>
       <c r="J24" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E25" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F25" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G25" t="s">
         <v>12</v>
       </c>
       <c r="H25" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="I25" t="s">
         <v>12</v>
       </c>
       <c r="J25" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -1895,62 +2090,62 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
+        <v>50</v>
+      </c>
+      <c r="H26" t="s">
+        <v>145</v>
+      </c>
+      <c r="I26" t="s">
         <v>57</v>
       </c>
-      <c r="H26" t="s">
-        <v>130</v>
-      </c>
-      <c r="I26" t="s">
-        <v>131</v>
-      </c>
       <c r="J26" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D27" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E27" t="s">
+        <v>147</v>
+      </c>
+      <c r="F27" t="s">
         <v>133</v>
       </c>
-      <c r="F27" t="s">
-        <v>51</v>
-      </c>
       <c r="G27" t="s">
         <v>12</v>
       </c>
       <c r="H27" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
       </c>
       <c r="J27" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -1959,62 +2154,62 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H28" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="I28" t="s">
-        <v>139</v>
+        <v>62</v>
       </c>
       <c r="J28" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B29" t="s">
         <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E29" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="F29" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G29" t="s">
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2023,62 +2218,62 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H30" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="I30" t="s">
-        <v>147</v>
+        <v>67</v>
       </c>
       <c r="J30" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B31" t="s">
         <v>12</v>
       </c>
       <c r="C31" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D31" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E31" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="F31" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G31" t="s">
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="I31" t="s">
         <v>12</v>
       </c>
       <c r="J31" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2087,62 +2282,62 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H32" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="I32" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="J32" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="B33" t="s">
         <v>12</v>
       </c>
       <c r="C33" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D33" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="F33" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G33" t="s">
         <v>12</v>
       </c>
       <c r="H33" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="I33" t="s">
         <v>12</v>
       </c>
       <c r="J33" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B34" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2151,62 +2346,62 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H34" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="I34" t="s">
-        <v>163</v>
+        <v>77</v>
       </c>
       <c r="J34" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="B35" t="s">
         <v>12</v>
       </c>
       <c r="C35" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D35" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E35" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="F35" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G35" t="s">
         <v>12</v>
       </c>
       <c r="H35" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="I35" t="s">
         <v>12</v>
       </c>
       <c r="J35" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2215,62 +2410,62 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H36" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="I36" t="s">
-        <v>171</v>
+        <v>82</v>
       </c>
       <c r="J36" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="B37" t="s">
         <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D37" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="F37" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G37" t="s">
         <v>12</v>
       </c>
       <c r="H37" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="I37" t="s">
         <v>12</v>
       </c>
       <c r="J37" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2279,62 +2474,62 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H38" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="I38" t="s">
-        <v>179</v>
+        <v>87</v>
       </c>
       <c r="J38" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B39" t="s">
         <v>12</v>
       </c>
       <c r="C39" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D39" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E39" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="F39" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G39" t="s">
         <v>12</v>
       </c>
       <c r="H39" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="I39" t="s">
         <v>12</v>
       </c>
       <c r="J39" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B40" t="s">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2343,62 +2538,62 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>187</v>
+        <v>50</v>
       </c>
       <c r="H40" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="I40" t="s">
-        <v>189</v>
+        <v>92</v>
       </c>
       <c r="J40" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
       </c>
       <c r="C41" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E41" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="F41" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G41" t="s">
         <v>12</v>
       </c>
       <c r="H41" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="I41" t="s">
         <v>12</v>
       </c>
       <c r="J41" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B42" t="s">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2407,62 +2602,62 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>187</v>
+        <v>50</v>
       </c>
       <c r="H42" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="I42" t="s">
-        <v>197</v>
+        <v>97</v>
       </c>
       <c r="J42" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B43" t="s">
         <v>12</v>
       </c>
       <c r="C43" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E43" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F43" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G43" t="s">
         <v>12</v>
       </c>
       <c r="H43" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I43" t="s">
         <v>12</v>
       </c>
       <c r="J43" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B44" t="s">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -2471,62 +2666,62 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>187</v>
+        <v>50</v>
       </c>
       <c r="H44" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="I44" t="s">
+        <v>102</v>
+      </c>
+      <c r="J44" t="s">
         <v>205</v>
-      </c>
-      <c r="J44" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E45" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F45" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G45" t="s">
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
       </c>
       <c r="J45" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B46" t="s">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -2535,62 +2730,62 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>187</v>
+        <v>50</v>
       </c>
       <c r="H46" t="s">
+        <v>215</v>
+      </c>
+      <c r="I46" t="s">
+        <v>107</v>
+      </c>
+      <c r="J46" t="s">
         <v>212</v>
-      </c>
-      <c r="I46" t="s">
-        <v>213</v>
-      </c>
-      <c r="J46" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B47" t="s">
         <v>12</v>
       </c>
       <c r="C47" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="E47" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F47" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="G47" t="s">
         <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I47" t="s">
         <v>12</v>
       </c>
       <c r="J47" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B48" t="s">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C48" t="s">
         <v>12</v>
@@ -2599,22 +2794,534 @@
         <v>12</v>
       </c>
       <c r="E48" t="s">
+        <v>221</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" t="s">
+        <v>222</v>
+      </c>
+      <c r="I48" t="s">
+        <v>112</v>
+      </c>
+      <c r="J48" t="s">
         <v>219</v>
       </c>
-      <c r="F48" t="s">
-        <v>14</v>
-      </c>
-      <c r="G48" t="s">
-        <v>187</v>
-      </c>
-      <c r="H48" t="s">
-        <v>220</v>
-      </c>
-      <c r="I48" t="s">
-        <v>221</v>
-      </c>
-      <c r="J48" t="s">
-        <v>217</v>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>223</v>
+      </c>
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" t="s">
+        <v>130</v>
+      </c>
+      <c r="D49" t="s">
+        <v>131</v>
+      </c>
+      <c r="E49" t="s">
+        <v>224</v>
+      </c>
+      <c r="F49" t="s">
+        <v>133</v>
+      </c>
+      <c r="G49" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" t="s">
+        <v>225</v>
+      </c>
+      <c r="I49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>227</v>
+      </c>
+      <c r="B50" t="s">
+        <v>48</v>
+      </c>
+      <c r="C50" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>228</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>50</v>
+      </c>
+      <c r="H50" t="s">
+        <v>229</v>
+      </c>
+      <c r="I50" t="s">
+        <v>117</v>
+      </c>
+      <c r="J50" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>230</v>
+      </c>
+      <c r="B51" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" t="s">
+        <v>130</v>
+      </c>
+      <c r="D51" t="s">
+        <v>131</v>
+      </c>
+      <c r="E51" t="s">
+        <v>231</v>
+      </c>
+      <c r="F51" t="s">
+        <v>133</v>
+      </c>
+      <c r="G51" t="s">
+        <v>12</v>
+      </c>
+      <c r="H51" t="s">
+        <v>232</v>
+      </c>
+      <c r="I51" t="s">
+        <v>12</v>
+      </c>
+      <c r="J51" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>234</v>
+      </c>
+      <c r="B52" t="s">
+        <v>48</v>
+      </c>
+      <c r="C52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>235</v>
+      </c>
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" t="s">
+        <v>50</v>
+      </c>
+      <c r="H52" t="s">
+        <v>236</v>
+      </c>
+      <c r="I52" t="s">
+        <v>122</v>
+      </c>
+      <c r="J52" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>237</v>
+      </c>
+      <c r="B53" t="s">
+        <v>12</v>
+      </c>
+      <c r="C53" t="s">
+        <v>130</v>
+      </c>
+      <c r="D53" t="s">
+        <v>131</v>
+      </c>
+      <c r="E53" t="s">
+        <v>238</v>
+      </c>
+      <c r="F53" t="s">
+        <v>133</v>
+      </c>
+      <c r="G53" t="s">
+        <v>12</v>
+      </c>
+      <c r="H53" t="s">
+        <v>239</v>
+      </c>
+      <c r="I53" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>241</v>
+      </c>
+      <c r="B54" t="s">
+        <v>48</v>
+      </c>
+      <c r="C54" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>242</v>
+      </c>
+      <c r="F54" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" t="s">
+        <v>50</v>
+      </c>
+      <c r="H54" t="s">
+        <v>243</v>
+      </c>
+      <c r="I54" t="s">
+        <v>127</v>
+      </c>
+      <c r="J54" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>244</v>
+      </c>
+      <c r="B55" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" t="s">
+        <v>130</v>
+      </c>
+      <c r="D55" t="s">
+        <v>131</v>
+      </c>
+      <c r="E55" t="s">
+        <v>245</v>
+      </c>
+      <c r="F55" t="s">
+        <v>133</v>
+      </c>
+      <c r="G55" t="s">
+        <v>12</v>
+      </c>
+      <c r="H55" t="s">
+        <v>246</v>
+      </c>
+      <c r="I55" t="s">
+        <v>12</v>
+      </c>
+      <c r="J55" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>248</v>
+      </c>
+      <c r="B56" t="s">
+        <v>249</v>
+      </c>
+      <c r="C56" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>250</v>
+      </c>
+      <c r="F56" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" t="s">
+        <v>251</v>
+      </c>
+      <c r="H56" t="s">
+        <v>252</v>
+      </c>
+      <c r="I56" t="s">
+        <v>253</v>
+      </c>
+      <c r="J56" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>254</v>
+      </c>
+      <c r="B57" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" t="s">
+        <v>130</v>
+      </c>
+      <c r="D57" t="s">
+        <v>131</v>
+      </c>
+      <c r="E57" t="s">
+        <v>255</v>
+      </c>
+      <c r="F57" t="s">
+        <v>133</v>
+      </c>
+      <c r="G57" t="s">
+        <v>12</v>
+      </c>
+      <c r="H57" t="s">
+        <v>256</v>
+      </c>
+      <c r="I57" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>258</v>
+      </c>
+      <c r="B58" t="s">
+        <v>249</v>
+      </c>
+      <c r="C58" t="s">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>259</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
+        <v>251</v>
+      </c>
+      <c r="H58" t="s">
+        <v>260</v>
+      </c>
+      <c r="I58" t="s">
+        <v>261</v>
+      </c>
+      <c r="J58" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>262</v>
+      </c>
+      <c r="B59" t="s">
+        <v>12</v>
+      </c>
+      <c r="C59" t="s">
+        <v>130</v>
+      </c>
+      <c r="D59" t="s">
+        <v>131</v>
+      </c>
+      <c r="E59" t="s">
+        <v>263</v>
+      </c>
+      <c r="F59" t="s">
+        <v>133</v>
+      </c>
+      <c r="G59" t="s">
+        <v>12</v>
+      </c>
+      <c r="H59" t="s">
+        <v>264</v>
+      </c>
+      <c r="I59" t="s">
+        <v>12</v>
+      </c>
+      <c r="J59" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>266</v>
+      </c>
+      <c r="B60" t="s">
+        <v>267</v>
+      </c>
+      <c r="C60" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>268</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>251</v>
+      </c>
+      <c r="H60" t="s">
+        <v>269</v>
+      </c>
+      <c r="I60" t="s">
+        <v>270</v>
+      </c>
+      <c r="J60" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>271</v>
+      </c>
+      <c r="B61" t="s">
+        <v>12</v>
+      </c>
+      <c r="C61" t="s">
+        <v>130</v>
+      </c>
+      <c r="D61" t="s">
+        <v>131</v>
+      </c>
+      <c r="E61" t="s">
+        <v>272</v>
+      </c>
+      <c r="F61" t="s">
+        <v>133</v>
+      </c>
+      <c r="G61" t="s">
+        <v>12</v>
+      </c>
+      <c r="H61" t="s">
+        <v>273</v>
+      </c>
+      <c r="I61" t="s">
+        <v>12</v>
+      </c>
+      <c r="J61" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>275</v>
+      </c>
+      <c r="B62" t="s">
+        <v>249</v>
+      </c>
+      <c r="C62" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>276</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>251</v>
+      </c>
+      <c r="H62" t="s">
+        <v>277</v>
+      </c>
+      <c r="I62" t="s">
+        <v>278</v>
+      </c>
+      <c r="J62" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>279</v>
+      </c>
+      <c r="B63" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" t="s">
+        <v>130</v>
+      </c>
+      <c r="D63" t="s">
+        <v>131</v>
+      </c>
+      <c r="E63" t="s">
+        <v>280</v>
+      </c>
+      <c r="F63" t="s">
+        <v>133</v>
+      </c>
+      <c r="G63" t="s">
+        <v>12</v>
+      </c>
+      <c r="H63" t="s">
+        <v>281</v>
+      </c>
+      <c r="I63" t="s">
+        <v>12</v>
+      </c>
+      <c r="J63" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>283</v>
+      </c>
+      <c r="B64" t="s">
+        <v>249</v>
+      </c>
+      <c r="C64" t="s">
+        <v>12</v>
+      </c>
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" t="s">
+        <v>284</v>
+      </c>
+      <c r="F64" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" t="s">
+        <v>251</v>
+      </c>
+      <c r="H64" t="s">
+        <v>285</v>
+      </c>
+      <c r="I64" t="s">
+        <v>286</v>
+      </c>
+      <c r="J64" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add author-bio block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 19
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-detail.report.xlsx
+++ b/tools/importer/reports/import-article-detail.report.xlsx
@@ -412,7 +412,7 @@
     <t>article-detail</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:11.279Z</t>
+    <t>2026-09-18T18:26:04.895Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -427,7 +427,7 @@
     <t>ca/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:16.735Z</t>
+    <t>2026-09-18T18:26:09.889Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -445,7 +445,7 @@
     <t>ca/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:31.488Z</t>
+    <t>2026-09-18T18:26:24.548Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -460,7 +460,7 @@
     <t>ca/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:36.895Z</t>
+    <t>2026-09-18T18:26:30.433Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -475,7 +475,7 @@
     <t>ca/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:41.821Z</t>
+    <t>2026-09-18T18:26:36.516Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -853,7 +853,7 @@
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:46.708Z</t>
+    <t>2026-09-18T18:26:41.149Z</t>
   </si>
   <si>
     <t>us/en/magazine/guide-la-skateparks.html.report.json</t>
@@ -874,7 +874,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:51.841Z</t>
+    <t>2026-09-18T18:26:48.052Z</t>
   </si>
   <si>
     <t>us/en/magazine/san-diego-surf.html.report.json</t>
@@ -895,7 +895,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:56.559Z</t>
+    <t>2026-09-18T18:26:54.021Z</t>
   </si>
   <si>
     <t>us/en/magazine/ski-touring.html.report.json</t>
@@ -916,7 +916,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-18T18:12:01.705Z</t>
+    <t>2026-09-18T18:26:58.809Z</t>
   </si>
   <si>
     <t>us/en/magazine/western-australia.html.report.json</t>
@@ -937,7 +937,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-18T18:12:07.973Z</t>
+    <t>2026-09-18T18:27:04.913Z</t>
   </si>
   <si>
     <t>ca/en/magazine/members-only/alaskan-adventure.report.json</t>
@@ -946,7 +946,7 @@
     <t>ca/en/magazine/members-only/alaskan-adventure</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:21.031Z</t>
+    <t>2026-09-18T18:26:15.345Z</t>
   </si>
   <si>
     <t>Alaskan Adventure</t>
@@ -961,7 +961,7 @@
     <t>ca/en/magazine/members-only/fly-fishing-the-amazon</t>
   </si>
   <si>
-    <t>2026-09-18T18:11:25.637Z</t>
+    <t>2026-09-18T18:26:19.855Z</t>
   </si>
   <si>
     <t>Fly Fishing the Amazon</t>

</xml_diff>